<commit_message>
chore(docs): update edt progress columns based on repo state
</commit_message>
<xml_diff>
--- a/docs/entrega_2/edt_entrega_2.xlsx
+++ b/docs/entrega_2/edt_entrega_2.xlsx
@@ -16,8 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="DD-MM-YYYY"/>
+    <numFmt numFmtId="165" formatCode="0&quot;%&quot;"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -56,7 +57,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -93,6 +94,11 @@
         <fgColor rgb="00D6E4BC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4CCCC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -120,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -182,6 +188,24 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -674,13 +698,13 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H4" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" s="5" t="n">
+      <c r="H4" s="23" t="n">
+        <v>100</v>
+      </c>
+      <c r="I4" s="23" t="n">
+        <v>100</v>
+      </c>
+      <c r="J4" s="23" t="n">
         <v>0</v>
       </c>
       <c r="K4" s="5" t="n">
@@ -720,13 +744,13 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H5" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="8" t="n">
+      <c r="H5" s="24" t="n">
+        <v>100</v>
+      </c>
+      <c r="I5" s="24" t="n">
+        <v>100</v>
+      </c>
+      <c r="J5" s="24" t="n">
         <v>0</v>
       </c>
       <c r="K5" s="8" t="n">
@@ -766,13 +790,13 @@
           <t>1.1</t>
         </is>
       </c>
-      <c r="H6" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="11" t="n">
+      <c r="H6" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="I6" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="J6" s="25" t="n">
         <v>0</v>
       </c>
       <c r="K6" s="11" t="n">
@@ -812,13 +836,13 @@
           <t>1.2</t>
         </is>
       </c>
-      <c r="H7" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="8" t="n">
+      <c r="H7" s="24" t="n">
+        <v>100</v>
+      </c>
+      <c r="I7" s="24" t="n">
+        <v>100</v>
+      </c>
+      <c r="J7" s="24" t="n">
         <v>0</v>
       </c>
       <c r="K7" s="8" t="n">
@@ -862,13 +886,13 @@
           <t>1.3</t>
         </is>
       </c>
-      <c r="H8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="5" t="n">
+      <c r="H8" s="23" t="n">
+        <v>100</v>
+      </c>
+      <c r="I8" s="23" t="n">
+        <v>100</v>
+      </c>
+      <c r="J8" s="23" t="n">
         <v>0</v>
       </c>
       <c r="K8" s="5" t="n">
@@ -908,13 +932,13 @@
           <t>1.3</t>
         </is>
       </c>
-      <c r="H9" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" s="8" t="n">
+      <c r="H9" s="24" t="n">
+        <v>100</v>
+      </c>
+      <c r="I9" s="24" t="n">
+        <v>100</v>
+      </c>
+      <c r="J9" s="24" t="n">
         <v>0</v>
       </c>
       <c r="K9" s="8" t="n">
@@ -954,13 +978,13 @@
           <t>2.1</t>
         </is>
       </c>
-      <c r="H10" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="11" t="n">
+      <c r="H10" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="I10" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="J10" s="25" t="n">
         <v>0</v>
       </c>
       <c r="K10" s="11" t="n">
@@ -1000,13 +1024,13 @@
           <t>2.2</t>
         </is>
       </c>
-      <c r="H11" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="14" t="n">
+      <c r="H11" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="I11" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="J11" s="26" t="n">
         <v>0</v>
       </c>
       <c r="K11" s="14" t="n">
@@ -1050,13 +1074,13 @@
           <t>2.3</t>
         </is>
       </c>
-      <c r="H12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" s="5" t="n">
+      <c r="H12" s="23" t="n">
+        <v>100</v>
+      </c>
+      <c r="I12" s="23" t="n">
+        <v>100</v>
+      </c>
+      <c r="J12" s="23" t="n">
         <v>0</v>
       </c>
       <c r="K12" s="5" t="n">
@@ -1096,13 +1120,13 @@
           <t>2.3</t>
         </is>
       </c>
-      <c r="H13" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="8" t="n">
+      <c r="H13" s="24" t="n">
+        <v>100</v>
+      </c>
+      <c r="I13" s="24" t="n">
+        <v>100</v>
+      </c>
+      <c r="J13" s="24" t="n">
         <v>0</v>
       </c>
       <c r="K13" s="8" t="n">
@@ -1142,13 +1166,13 @@
           <t>2.3</t>
         </is>
       </c>
-      <c r="H14" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="11" t="n">
+      <c r="H14" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="I14" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="J14" s="25" t="n">
         <v>0</v>
       </c>
       <c r="K14" s="11" t="n">
@@ -1188,13 +1212,13 @@
           <t>3.2</t>
         </is>
       </c>
-      <c r="H15" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="8" t="n">
+      <c r="H15" s="24" t="n">
+        <v>100</v>
+      </c>
+      <c r="I15" s="24" t="n">
+        <v>100</v>
+      </c>
+      <c r="J15" s="24" t="n">
         <v>0</v>
       </c>
       <c r="K15" s="8" t="n">
@@ -1234,13 +1258,13 @@
           <t>3.3</t>
         </is>
       </c>
-      <c r="H16" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="11" t="n">
+      <c r="H16" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="I16" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="J16" s="25" t="n">
         <v>0</v>
       </c>
       <c r="K16" s="11" t="n">
@@ -1280,13 +1304,13 @@
           <t>3.4</t>
         </is>
       </c>
-      <c r="H17" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" s="14" t="n">
+      <c r="H17" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="I17" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="J17" s="26" t="n">
         <v>0</v>
       </c>
       <c r="K17" s="14" t="n">
@@ -1330,14 +1354,14 @@
           <t>3.5</t>
         </is>
       </c>
-      <c r="H18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" s="5" t="n">
-        <v>0</v>
+      <c r="H18" s="23" t="n">
+        <v>100</v>
+      </c>
+      <c r="I18" s="23" t="n">
+        <v>69</v>
+      </c>
+      <c r="J18" s="27" t="n">
+        <v>-31</v>
       </c>
       <c r="K18" s="5" t="n">
         <v>88</v>
@@ -1376,13 +1400,13 @@
           <t>3.5</t>
         </is>
       </c>
-      <c r="H19" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="8" t="n">
+      <c r="H19" s="24" t="n">
+        <v>100</v>
+      </c>
+      <c r="I19" s="24" t="n">
+        <v>100</v>
+      </c>
+      <c r="J19" s="24" t="n">
         <v>0</v>
       </c>
       <c r="K19" s="8" t="n">
@@ -1422,13 +1446,13 @@
           <t>4.1</t>
         </is>
       </c>
-      <c r="H20" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" s="11" t="n">
+      <c r="H20" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="I20" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="J20" s="25" t="n">
         <v>0</v>
       </c>
       <c r="K20" s="11" t="n">
@@ -1468,13 +1492,13 @@
           <t>4.2</t>
         </is>
       </c>
-      <c r="H21" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J21" s="8" t="n">
+      <c r="H21" s="24" t="n">
+        <v>100</v>
+      </c>
+      <c r="I21" s="24" t="n">
+        <v>100</v>
+      </c>
+      <c r="J21" s="24" t="n">
         <v>0</v>
       </c>
       <c r="K21" s="8" t="n">
@@ -1514,13 +1538,13 @@
           <t>3.5</t>
         </is>
       </c>
-      <c r="H22" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I22" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J22" s="11" t="n">
+      <c r="H22" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="I22" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="J22" s="25" t="n">
         <v>0</v>
       </c>
       <c r="K22" s="11" t="n">
@@ -1560,14 +1584,14 @@
           <t>4.4</t>
         </is>
       </c>
-      <c r="H23" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" s="8" t="n">
-        <v>0</v>
+      <c r="H23" s="24" t="n">
+        <v>100</v>
+      </c>
+      <c r="I23" s="24" t="n">
+        <v>60</v>
+      </c>
+      <c r="J23" s="28" t="n">
+        <v>-40</v>
       </c>
       <c r="K23" s="8" t="n">
         <v>8</v>
@@ -1606,14 +1630,14 @@
           <t>4.5</t>
         </is>
       </c>
-      <c r="H24" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" s="11" t="n">
-        <v>0</v>
+      <c r="H24" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="I24" s="25" t="n">
+        <v>50</v>
+      </c>
+      <c r="J24" s="28" t="n">
+        <v>-50</v>
       </c>
       <c r="K24" s="11" t="n">
         <v>24</v>
@@ -1652,14 +1676,14 @@
           <t>4.6</t>
         </is>
       </c>
-      <c r="H25" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I25" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J25" s="8" t="n">
-        <v>0</v>
+      <c r="H25" s="24" t="n">
+        <v>100</v>
+      </c>
+      <c r="I25" s="24" t="n">
+        <v>50</v>
+      </c>
+      <c r="J25" s="28" t="n">
+        <v>-50</v>
       </c>
       <c r="K25" s="8" t="n">
         <v>8</v>
@@ -1698,14 +1722,14 @@
           <t>4.7</t>
         </is>
       </c>
-      <c r="H26" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I26" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J26" s="11" t="n">
-        <v>0</v>
+      <c r="H26" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="I26" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="28" t="n">
+        <v>-100</v>
       </c>
       <c r="K26" s="11" t="n">
         <v>8</v>
@@ -1748,13 +1772,13 @@
           <t>4.8</t>
         </is>
       </c>
-      <c r="H27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" s="5" t="n">
+      <c r="H27" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="23" t="n">
         <v>0</v>
       </c>
       <c r="K27" s="5" t="n">
@@ -1794,13 +1818,13 @@
           <t>4.8</t>
         </is>
       </c>
-      <c r="H28" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I28" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J28" s="11" t="n">
+      <c r="H28" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="25" t="n">
         <v>0</v>
       </c>
       <c r="K28" s="11" t="n">
@@ -1840,13 +1864,13 @@
           <t>5.1</t>
         </is>
       </c>
-      <c r="H29" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I29" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J29" s="8" t="n">
+      <c r="H29" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="24" t="n">
         <v>0</v>
       </c>
       <c r="K29" s="8" t="n">
@@ -1886,13 +1910,13 @@
           <t>5.2</t>
         </is>
       </c>
-      <c r="H30" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I30" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J30" s="11" t="n">
+      <c r="H30" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="25" t="n">
         <v>0</v>
       </c>
       <c r="K30" s="11" t="n">
@@ -1932,13 +1956,13 @@
           <t>5.3</t>
         </is>
       </c>
-      <c r="H31" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I31" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J31" s="8" t="n">
+      <c r="H31" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="24" t="n">
         <v>0</v>
       </c>
       <c r="K31" s="8" t="n">
@@ -1978,13 +2002,13 @@
           <t>5.4</t>
         </is>
       </c>
-      <c r="H32" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I32" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J32" s="11" t="n">
+      <c r="H32" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" s="25" t="n">
         <v>0</v>
       </c>
       <c r="K32" s="11" t="n">
@@ -2024,13 +2048,13 @@
           <t>5.5</t>
         </is>
       </c>
-      <c r="H33" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I33" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J33" s="8" t="n">
+      <c r="H33" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" s="24" t="n">
         <v>0</v>
       </c>
       <c r="K33" s="8" t="n">
@@ -2070,13 +2094,13 @@
           <t>5.6</t>
         </is>
       </c>
-      <c r="H34" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I34" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J34" s="14" t="n">
+      <c r="H34" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" s="26" t="n">
         <v>0</v>
       </c>
       <c r="K34" s="14" t="n">
@@ -2120,13 +2144,13 @@
           <t>5.7</t>
         </is>
       </c>
-      <c r="H35" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I35" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J35" s="5" t="n">
+      <c r="H35" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" s="23" t="n">
         <v>0</v>
       </c>
       <c r="K35" s="5" t="n">
@@ -2166,13 +2190,13 @@
           <t>5.7</t>
         </is>
       </c>
-      <c r="H36" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I36" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J36" s="11" t="n">
+      <c r="H36" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" s="25" t="n">
         <v>0</v>
       </c>
       <c r="K36" s="11" t="n">
@@ -2212,13 +2236,13 @@
           <t>6.1</t>
         </is>
       </c>
-      <c r="H37" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I37" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J37" s="8" t="n">
+      <c r="H37" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" s="24" t="n">
         <v>0</v>
       </c>
       <c r="K37" s="8" t="n">
@@ -2258,13 +2282,13 @@
           <t>6.2</t>
         </is>
       </c>
-      <c r="H38" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I38" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J38" s="11" t="n">
+      <c r="H38" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" s="25" t="n">
         <v>0</v>
       </c>
       <c r="K38" s="11" t="n">
@@ -2308,13 +2332,13 @@
           <t>6.3</t>
         </is>
       </c>
-      <c r="H39" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I39" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J39" s="5" t="n">
+      <c r="H39" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" s="23" t="n">
         <v>0</v>
       </c>
       <c r="K39" s="5" t="n">
@@ -2354,13 +2378,13 @@
           <t>6.3</t>
         </is>
       </c>
-      <c r="H40" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I40" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J40" s="11" t="n">
+      <c r="H40" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J40" s="25" t="n">
         <v>0</v>
       </c>
       <c r="K40" s="11" t="n">
@@ -2400,13 +2424,13 @@
           <t>7.1</t>
         </is>
       </c>
-      <c r="H41" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I41" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J41" s="8" t="n">
+      <c r="H41" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" s="24" t="n">
         <v>0</v>
       </c>
       <c r="K41" s="8" t="n">
@@ -2450,13 +2474,13 @@
           <t>7.2</t>
         </is>
       </c>
-      <c r="H42" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I42" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J42" s="5" t="n">
+      <c r="H42" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="J42" s="23" t="n">
         <v>0</v>
       </c>
       <c r="K42" s="5" t="n">
@@ -2496,13 +2520,13 @@
           <t>7.2</t>
         </is>
       </c>
-      <c r="H43" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I43" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J43" s="8" t="n">
+      <c r="H43" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" s="24" t="n">
         <v>0</v>
       </c>
       <c r="K43" s="8" t="n">
@@ -2542,13 +2566,13 @@
           <t>8.1</t>
         </is>
       </c>
-      <c r="H44" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I44" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J44" s="14" t="n">
+      <c r="H44" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" s="26" t="n">
         <v>0</v>
       </c>
       <c r="K44" s="14" t="n">

</xml_diff>